<commit_message>
GRNLED extract: cleaner beam angles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011z5jzBt752B8P8p43rbdhg
</commit_message>
<xml_diff>
--- a/dimo-lighting-ops/data/catalogs/GRNLED_catalogue_extract.xlsx
+++ b/dimo-lighting-ops/data/catalogs/GRNLED_catalogue_extract.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
@@ -746,7 +746,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -833,7 +833,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -920,7 +920,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>15°/24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>15°/24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>15°/24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>15°/24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>15°/24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
@@ -1875,7 +1875,11 @@
       <c r="I16" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
@@ -1958,7 +1962,11 @@
       <c r="I17" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -2041,7 +2049,11 @@
       <c r="I18" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
@@ -2124,7 +2136,11 @@
       <c r="I19" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -2207,7 +2223,11 @@
       <c r="I20" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -2705,7 +2725,11 @@
       <c r="I26" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -2788,7 +2812,11 @@
       <c r="I27" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
@@ -2871,7 +2899,11 @@
       <c r="I28" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -2954,7 +2986,11 @@
       <c r="I29" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -5724,7 +5760,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/100°</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
@@ -5811,7 +5847,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/100°</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr"/>
@@ -5898,7 +5934,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/100°</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -5985,7 +6021,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/100°</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
@@ -6072,7 +6108,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/100°</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
@@ -6159,7 +6195,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/24°/100°</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
@@ -6246,7 +6282,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>120°</t>
+          <t>120°/24°/100°</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
@@ -6333,7 +6369,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>320°</t>
+          <t>320°/100°</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
@@ -6420,7 +6456,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>320°</t>
+          <t>320°/100°</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -9368,7 +9404,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -9471,7 +9507,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr">
@@ -9574,7 +9610,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -9677,7 +9713,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
@@ -9780,7 +9816,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -9883,7 +9919,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>24°36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -9986,7 +10022,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>24°36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -10089,7 +10125,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>24°36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K108" s="2" t="inlineStr">
@@ -10192,7 +10228,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>24°36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
@@ -10295,7 +10331,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>24°36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -10398,7 +10434,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr">
@@ -10501,7 +10537,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
@@ -10604,7 +10640,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr">
@@ -10707,7 +10743,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>15°24°36°50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -11531,7 +11567,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>24° 36° 60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K122" s="2" t="inlineStr">
@@ -11630,7 +11666,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>24° 36° 60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr">
@@ -11729,7 +11765,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>24° 36° 60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K124" s="2" t="inlineStr">
@@ -11828,7 +11864,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>24° 36° 60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K125" s="2" t="inlineStr">
@@ -11927,7 +11963,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>24° 36° 60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K126" s="2" t="inlineStr">
@@ -12026,7 +12062,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr"/>
@@ -12121,7 +12157,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K128" s="2" t="inlineStr"/>
@@ -12216,7 +12252,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K129" s="2" t="inlineStr"/>
@@ -12311,7 +12347,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K130" s="2" t="inlineStr"/>
@@ -12406,7 +12442,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr"/>
@@ -12996,7 +13032,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -13095,7 +13131,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr">
@@ -13194,7 +13230,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
@@ -13293,7 +13329,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K140" s="2" t="inlineStr">
@@ -13392,7 +13428,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K141" s="2" t="inlineStr">
@@ -14677,7 +14713,11 @@
       <c r="I154" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -14772,7 +14812,11 @@
       <c r="I155" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J155" s="2" t="inlineStr"/>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K155" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -14867,7 +14911,11 @@
       <c r="I156" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -14962,7 +15010,11 @@
       <c r="I157" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J157" s="2" t="inlineStr"/>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -15057,7 +15109,11 @@
       <c r="I158" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K158" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -15152,7 +15208,11 @@
       <c r="I159" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J159" s="2" t="inlineStr"/>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K159" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -16534,7 +16594,11 @@
       <c r="I173" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -16629,7 +16693,11 @@
       <c r="I174" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K174" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -16724,7 +16792,11 @@
       <c r="I175" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K175" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -16819,7 +16891,11 @@
       <c r="I176" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K176" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -16914,7 +16990,11 @@
       <c r="I177" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K177" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17009,7 +17089,11 @@
       <c r="I178" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>60°/90°</t>
+        </is>
+      </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17104,7 +17188,11 @@
       <c r="I179" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K179" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17199,7 +17287,11 @@
       <c r="I180" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K180" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17294,7 +17386,11 @@
       <c r="I181" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K181" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17389,7 +17485,11 @@
       <c r="I182" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K182" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17484,7 +17584,11 @@
       <c r="I183" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="J183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K183" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -17579,7 +17683,11 @@
       <c r="I184" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K184" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -17678,7 +17786,11 @@
       <c r="I185" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K185" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -17777,7 +17889,11 @@
       <c r="I186" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -17876,7 +17992,11 @@
       <c r="I187" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="J187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K187" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -17975,7 +18095,11 @@
       <c r="I188" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -18074,7 +18198,11 @@
       <c r="I189" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="J189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>36°/60°</t>
+        </is>
+      </c>
       <c r="K189" s="2" t="inlineStr">
         <is>
           <t>IP20–11</t>
@@ -18169,7 +18297,11 @@
       <c r="I190" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J190" s="2" t="inlineStr"/>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -18260,7 +18392,11 @@
       <c r="I191" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -18351,7 +18487,11 @@
       <c r="I192" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J192" s="2" t="inlineStr"/>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -18442,7 +18582,11 @@
       <c r="I193" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -18931,7 +19075,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>24°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr">
@@ -19030,7 +19174,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>24°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -19129,7 +19273,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>24°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -19228,7 +19372,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>24°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -19329,7 +19473,11 @@
       <c r="I202" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19424,7 +19572,11 @@
       <c r="I203" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19519,7 +19671,11 @@
       <c r="I204" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J204" s="2" t="inlineStr"/>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19614,7 +19770,11 @@
       <c r="I205" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="J205" s="2" t="inlineStr"/>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K205" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19709,7 +19869,11 @@
       <c r="I206" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J206" s="2" t="inlineStr"/>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K206" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19804,7 +19968,11 @@
       <c r="I207" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J207" s="2" t="inlineStr"/>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19899,7 +20067,11 @@
       <c r="I208" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J208" s="2" t="inlineStr"/>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K208" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -19994,7 +20166,11 @@
       <c r="I209" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J209" s="2" t="inlineStr"/>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20089,7 +20265,11 @@
       <c r="I210" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J210" s="2" t="inlineStr"/>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K210" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20184,7 +20364,11 @@
       <c r="I211" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J211" s="2" t="inlineStr"/>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K211" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20279,7 +20463,11 @@
       <c r="I212" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J212" s="2" t="inlineStr"/>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20374,7 +20562,11 @@
       <c r="I213" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J213" s="2" t="inlineStr"/>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20469,7 +20661,11 @@
       <c r="I214" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J214" s="2" t="inlineStr"/>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20564,7 +20760,11 @@
       <c r="I215" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J215" s="2" t="inlineStr"/>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -20659,7 +20859,11 @@
       <c r="I216" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J216" s="2" t="inlineStr"/>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -20754,7 +20958,11 @@
       <c r="I217" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J217" s="2" t="inlineStr"/>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -20849,7 +21057,11 @@
       <c r="I218" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J218" s="2" t="inlineStr"/>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -20944,7 +21156,11 @@
       <c r="I219" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J219" s="2" t="inlineStr"/>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21035,7 +21251,11 @@
       <c r="I220" s="5" t="n">
         <v>1400</v>
       </c>
-      <c r="J220" s="2" t="inlineStr"/>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21126,7 +21346,11 @@
       <c r="I221" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J221" s="2" t="inlineStr"/>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21217,7 +21441,11 @@
       <c r="I222" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J222" s="2" t="inlineStr"/>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21308,7 +21536,11 @@
       <c r="I223" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J223" s="2" t="inlineStr"/>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K223" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21399,7 +21631,11 @@
       <c r="I224" s="5" t="n">
         <v>2100</v>
       </c>
-      <c r="J224" s="2" t="inlineStr"/>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21490,7 +21726,11 @@
       <c r="I225" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J225" s="2" t="inlineStr"/>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21581,7 +21821,11 @@
       <c r="I226" s="5" t="n">
         <v>4500</v>
       </c>
-      <c r="J226" s="2" t="inlineStr"/>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K226" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21672,7 +21916,11 @@
       <c r="I227" s="5" t="n">
         <v>6000</v>
       </c>
-      <c r="J227" s="2" t="inlineStr"/>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K227" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -21767,7 +22015,11 @@
       <c r="I228" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J228" s="2" t="inlineStr"/>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>15°–45° (adjustable)</t>
+        </is>
+      </c>
       <c r="K228" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -21862,7 +22114,11 @@
       <c r="I229" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J229" s="2" t="inlineStr"/>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>15°–45° (adjustable)</t>
+        </is>
+      </c>
       <c r="K229" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -21957,7 +22213,11 @@
       <c r="I230" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J230" s="2" t="inlineStr"/>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>15°–45° (adjustable)</t>
+        </is>
+      </c>
       <c r="K230" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22052,7 +22312,11 @@
       <c r="I231" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J231" s="2" t="inlineStr"/>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>15°–45° (adjustable)</t>
+        </is>
+      </c>
       <c r="K231" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22147,7 +22411,11 @@
       <c r="I232" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="J232" s="2" t="inlineStr"/>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>15°–45° (adjustable)</t>
+        </is>
+      </c>
       <c r="K232" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22242,7 +22510,11 @@
       <c r="I233" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J233" s="2" t="inlineStr"/>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K233" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22341,7 +22613,11 @@
       <c r="I234" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J234" s="2" t="inlineStr"/>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K234" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22440,7 +22716,11 @@
       <c r="I235" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J235" s="2" t="inlineStr"/>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K235" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22539,7 +22819,11 @@
       <c r="I236" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J236" s="2" t="inlineStr"/>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -22638,7 +22922,11 @@
       <c r="I237" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="J237" s="2" t="inlineStr"/>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°</t>
+        </is>
+      </c>
       <c r="K237" s="2" t="inlineStr">
         <is>
           <t>IP20</t>
@@ -23729,7 +24017,7 @@
       </c>
       <c r="J248" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K248" s="2" t="inlineStr">
@@ -23828,7 +24116,7 @@
       </c>
       <c r="J249" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K249" s="2" t="inlineStr">
@@ -23927,7 +24215,7 @@
       </c>
       <c r="J250" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K250" s="2" t="inlineStr">
@@ -24026,7 +24314,7 @@
       </c>
       <c r="J251" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K251" s="2" t="inlineStr">
@@ -25131,7 +25419,7 @@
       </c>
       <c r="J262" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°/55°</t>
+          <t>15°/24°/36°/55°</t>
         </is>
       </c>
       <c r="K262" s="2" t="inlineStr">
@@ -25234,7 +25522,7 @@
       </c>
       <c r="J263" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°/55°</t>
+          <t>15°/24°/36°/55°</t>
         </is>
       </c>
       <c r="K263" s="2" t="inlineStr">
@@ -25337,7 +25625,7 @@
       </c>
       <c r="J264" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°/55°</t>
+          <t>15°/24°/36°/55°</t>
         </is>
       </c>
       <c r="K264" s="2" t="inlineStr">
@@ -25749,7 +26037,7 @@
       </c>
       <c r="J268" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/55°</t>
         </is>
       </c>
       <c r="K268" s="2" t="inlineStr">
@@ -25856,7 +26144,7 @@
       </c>
       <c r="J269" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/55°</t>
         </is>
       </c>
       <c r="K269" s="2" t="inlineStr">
@@ -25963,7 +26251,7 @@
       </c>
       <c r="J270" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/55°</t>
         </is>
       </c>
       <c r="K270" s="2" t="inlineStr">
@@ -26066,7 +26354,7 @@
       </c>
       <c r="J271" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/50°</t>
         </is>
       </c>
       <c r="K271" s="2" t="inlineStr">
@@ -26165,7 +26453,7 @@
       </c>
       <c r="J272" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/50°</t>
         </is>
       </c>
       <c r="K272" s="2" t="inlineStr">
@@ -26264,7 +26552,7 @@
       </c>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/50°</t>
         </is>
       </c>
       <c r="K273" s="2" t="inlineStr">
@@ -26363,7 +26651,7 @@
       </c>
       <c r="J274" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/50°</t>
         </is>
       </c>
       <c r="K274" s="2" t="inlineStr">
@@ -26462,7 +26750,7 @@
       </c>
       <c r="J275" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>36°/50°</t>
         </is>
       </c>
       <c r="K275" s="2" t="inlineStr">
@@ -26565,7 +26853,7 @@
       </c>
       <c r="J276" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K276" s="2" t="inlineStr">
@@ -26668,7 +26956,7 @@
       </c>
       <c r="J277" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K277" s="2" t="inlineStr">
@@ -26771,7 +27059,7 @@
       </c>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K278" s="2" t="inlineStr">
@@ -26874,7 +27162,7 @@
       </c>
       <c r="J279" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K279" s="2" t="inlineStr">
@@ -26977,7 +27265,7 @@
       </c>
       <c r="J280" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K280" s="2" t="inlineStr">
@@ -27080,7 +27368,7 @@
       </c>
       <c r="J281" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K281" s="2" t="inlineStr">
@@ -27183,7 +27471,7 @@
       </c>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K282" s="2" t="inlineStr">
@@ -27286,7 +27574,7 @@
       </c>
       <c r="J283" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K283" s="2" t="inlineStr">
@@ -27389,7 +27677,7 @@
       </c>
       <c r="J284" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K284" s="2" t="inlineStr">
@@ -27492,7 +27780,7 @@
       </c>
       <c r="J285" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K285" s="2" t="inlineStr">
@@ -27595,7 +27883,7 @@
       </c>
       <c r="J286" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K286" s="2" t="inlineStr">
@@ -27698,7 +27986,7 @@
       </c>
       <c r="J287" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K287" s="2" t="inlineStr">
@@ -27797,7 +28085,7 @@
       </c>
       <c r="J288" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K288" s="2" t="inlineStr">
@@ -27896,7 +28184,7 @@
       </c>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K289" s="2" t="inlineStr">
@@ -27995,7 +28283,7 @@
       </c>
       <c r="J290" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K290" s="2" t="inlineStr">
@@ -28094,7 +28382,7 @@
       </c>
       <c r="J291" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/60°</t>
+          <t>15°/24°/36°/60°</t>
         </is>
       </c>
       <c r="K291" s="2" t="inlineStr">
@@ -28193,7 +28481,7 @@
       </c>
       <c r="J292" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K292" s="2" t="inlineStr">
@@ -28296,7 +28584,7 @@
       </c>
       <c r="J293" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K293" s="2" t="inlineStr">
@@ -28399,7 +28687,7 @@
       </c>
       <c r="J294" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K294" s="2" t="inlineStr">
@@ -28502,7 +28790,7 @@
       </c>
       <c r="J295" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K295" s="2" t="inlineStr">
@@ -28605,7 +28893,7 @@
       </c>
       <c r="J296" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K296" s="2" t="inlineStr">
@@ -28708,7 +28996,7 @@
       </c>
       <c r="J297" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K297" s="2" t="inlineStr">
@@ -28811,7 +29099,7 @@
       </c>
       <c r="J298" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K298" s="2" t="inlineStr">
@@ -28914,7 +29202,7 @@
       </c>
       <c r="J299" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K299" s="2" t="inlineStr">
@@ -29017,7 +29305,7 @@
       </c>
       <c r="J300" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K300" s="2" t="inlineStr">
@@ -29120,7 +29408,7 @@
       </c>
       <c r="J301" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K301" s="2" t="inlineStr">
@@ -29223,7 +29511,7 @@
       </c>
       <c r="J302" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K302" s="2" t="inlineStr">
@@ -29326,7 +29614,7 @@
       </c>
       <c r="J303" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K303" s="2" t="inlineStr">
@@ -29429,7 +29717,7 @@
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
@@ -29532,7 +29820,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr">
@@ -29631,7 +29919,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr">
@@ -29730,7 +30018,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr">
@@ -29829,7 +30117,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr">
@@ -29928,7 +30216,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr">
@@ -30300,7 +30588,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>25°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -30403,7 +30691,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>25°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -30506,7 +30794,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>25°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr">
@@ -30609,7 +30897,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>25°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr">
@@ -30712,7 +31000,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>25°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr">
@@ -30813,7 +31101,11 @@
       <c r="I318" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J318" s="2" t="inlineStr"/>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K318" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -30912,7 +31204,11 @@
       <c r="I319" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J319" s="2" t="inlineStr"/>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K319" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -31011,7 +31307,11 @@
       <c r="I320" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J320" s="2" t="inlineStr"/>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K320" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -31110,7 +31410,11 @@
       <c r="I321" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="J321" s="2" t="inlineStr"/>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -31209,7 +31513,11 @@
       <c r="I322" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J322" s="2" t="inlineStr"/>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -31310,7 +31618,7 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>36°/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K323" s="2" t="inlineStr">
@@ -31413,7 +31721,7 @@
       </c>
       <c r="J324" s="2" t="inlineStr">
         <is>
-          <t>36°/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K324" s="2" t="inlineStr">
@@ -31516,7 +31824,7 @@
       </c>
       <c r="J325" s="2" t="inlineStr">
         <is>
-          <t>36°/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K325" s="2" t="inlineStr">
@@ -31619,7 +31927,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>36°/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr">
@@ -31720,7 +32028,11 @@
       <c r="I327" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J327" s="2" t="inlineStr"/>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K327" s="2" t="inlineStr"/>
       <c r="L327" s="2" t="inlineStr">
         <is>
@@ -31807,7 +32119,11 @@
       <c r="I328" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J328" s="2" t="inlineStr"/>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K328" s="2" t="inlineStr"/>
       <c r="L328" s="2" t="inlineStr">
         <is>
@@ -31894,7 +32210,11 @@
       <c r="I329" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J329" s="2" t="inlineStr"/>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K329" s="2" t="inlineStr"/>
       <c r="L329" s="2" t="inlineStr">
         <is>
@@ -31981,7 +32301,11 @@
       <c r="I330" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="J330" s="2" t="inlineStr"/>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K330" s="2" t="inlineStr"/>
       <c r="L330" s="2" t="inlineStr">
         <is>
@@ -32068,7 +32392,11 @@
       <c r="I331" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J331" s="2" t="inlineStr"/>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K331" s="2" t="inlineStr"/>
       <c r="L331" s="2" t="inlineStr">
         <is>
@@ -32155,7 +32483,11 @@
       <c r="I332" s="5" t="n">
         <v>900</v>
       </c>
-      <c r="J332" s="2" t="inlineStr"/>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K332" s="2" t="inlineStr"/>
       <c r="L332" s="2" t="inlineStr">
         <is>
@@ -32242,7 +32574,11 @@
       <c r="I333" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J333" s="2" t="inlineStr"/>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>15°–60° (adjustable)</t>
+        </is>
+      </c>
       <c r="K333" s="2" t="inlineStr"/>
       <c r="L333" s="2" t="inlineStr">
         <is>
@@ -32331,7 +32667,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr">
@@ -32430,7 +32766,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr">
@@ -32529,7 +32865,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr">
@@ -32628,7 +32964,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>15/24/36/50°</t>
+          <t>15°/24°/36°/50°</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -32727,7 +33063,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -32826,7 +33162,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr">
@@ -32925,7 +33261,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr">
@@ -33024,7 +33360,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr">
@@ -33123,7 +33459,7 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr"/>
@@ -33218,7 +33554,7 @@
       </c>
       <c r="J343" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K343" s="2" t="inlineStr"/>
@@ -33313,7 +33649,7 @@
       </c>
       <c r="J344" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K344" s="2" t="inlineStr"/>
@@ -33408,7 +33744,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -34097,7 +34433,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr">
@@ -34196,7 +34532,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr">
@@ -34295,7 +34631,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -34394,7 +34730,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr">
@@ -34493,7 +34829,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -34592,7 +34928,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -34691,7 +35027,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -34790,7 +35126,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
@@ -34889,7 +35225,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -34988,7 +35324,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr">
@@ -35087,7 +35423,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr">
@@ -35186,7 +35522,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -35285,7 +35621,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr">
@@ -35384,7 +35720,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°/120°</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -35479,7 +35815,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°/120°</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
@@ -35574,7 +35910,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°/120°</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -35669,7 +36005,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>55°</t>
+          <t>24°/36°/55°</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr">
@@ -35772,7 +36108,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>55°</t>
+          <t>24°/36°/55°</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr">
@@ -35875,7 +36211,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr">
@@ -35978,7 +36314,7 @@
       </c>
       <c r="J371" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K371" s="2" t="inlineStr">
@@ -36081,7 +36417,7 @@
       </c>
       <c r="J372" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K372" s="2" t="inlineStr">
@@ -36184,7 +36520,7 @@
       </c>
       <c r="J373" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K373" s="2" t="inlineStr">
@@ -36283,7 +36619,7 @@
       </c>
       <c r="J374" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K374" s="2" t="inlineStr">
@@ -36382,7 +36718,7 @@
       </c>
       <c r="J375" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K375" s="2" t="inlineStr">
@@ -36481,7 +36817,7 @@
       </c>
       <c r="J376" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K376" s="2" t="inlineStr">
@@ -36580,7 +36916,7 @@
       </c>
       <c r="J377" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K377" s="2" t="inlineStr">
@@ -36679,7 +37015,7 @@
       </c>
       <c r="J378" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K378" s="2" t="inlineStr">
@@ -36776,7 +37112,11 @@
       <c r="I379" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J379" s="2" t="inlineStr"/>
+      <c r="J379" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K379" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -36875,7 +37215,11 @@
       <c r="I380" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J380" s="2" t="inlineStr"/>
+      <c r="J380" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K380" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -36974,7 +37318,11 @@
       <c r="I381" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J381" s="2" t="inlineStr"/>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K381" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -37073,7 +37421,11 @@
       <c r="I382" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J382" s="2" t="inlineStr"/>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K382" s="2" t="inlineStr">
         <is>
           <t>IP44</t>
@@ -37174,7 +37526,7 @@
       </c>
       <c r="J383" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K383" s="2" t="inlineStr">
@@ -37273,7 +37625,7 @@
       </c>
       <c r="J384" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K384" s="2" t="inlineStr">
@@ -37372,7 +37724,7 @@
       </c>
       <c r="J385" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K385" s="2" t="inlineStr">
@@ -37467,7 +37819,7 @@
       </c>
       <c r="J386" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K386" s="2" t="inlineStr">
@@ -37562,7 +37914,7 @@
       </c>
       <c r="J387" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K387" s="2" t="inlineStr">
@@ -37657,7 +38009,7 @@
       </c>
       <c r="J388" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K388" s="2" t="inlineStr">
@@ -37750,7 +38102,11 @@
       <c r="I389" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J389" s="2" t="inlineStr"/>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K389" s="2" t="inlineStr"/>
       <c r="L389" s="2" t="inlineStr">
         <is>
@@ -37837,7 +38193,11 @@
       <c r="I390" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J390" s="2" t="inlineStr"/>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K390" s="2" t="inlineStr"/>
       <c r="L390" s="2" t="inlineStr">
         <is>
@@ -37924,7 +38284,11 @@
       <c r="I391" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J391" s="2" t="inlineStr"/>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K391" s="2" t="inlineStr"/>
       <c r="L391" s="2" t="inlineStr">
         <is>
@@ -38011,7 +38375,11 @@
       <c r="I392" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J392" s="2" t="inlineStr"/>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K392" s="2" t="inlineStr"/>
       <c r="L392" s="2" t="inlineStr">
         <is>
@@ -38100,7 +38468,7 @@
       </c>
       <c r="J393" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K393" s="2" t="inlineStr">
@@ -38195,7 +38563,7 @@
       </c>
       <c r="J394" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K394" s="2" t="inlineStr">
@@ -38290,7 +38658,7 @@
       </c>
       <c r="J395" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K395" s="2" t="inlineStr">
@@ -38765,7 +39133,7 @@
       </c>
       <c r="J400" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K400" s="2" t="inlineStr">
@@ -38860,7 +39228,7 @@
       </c>
       <c r="J401" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K401" s="2" t="inlineStr">
@@ -38955,7 +39323,7 @@
       </c>
       <c r="J402" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K402" s="2" t="inlineStr">
@@ -39050,7 +39418,7 @@
       </c>
       <c r="J403" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K403" s="2" t="inlineStr">
@@ -39145,7 +39513,7 @@
       </c>
       <c r="J404" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K404" s="2" t="inlineStr">
@@ -39236,7 +39604,7 @@
       </c>
       <c r="J405" s="2" t="inlineStr">
         <is>
-          <t>24/36/60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K405" s="2" t="inlineStr">
@@ -39327,7 +39695,7 @@
       </c>
       <c r="J406" s="2" t="inlineStr">
         <is>
-          <t>24/36/60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K406" s="2" t="inlineStr">
@@ -39418,7 +39786,7 @@
       </c>
       <c r="J407" s="2" t="inlineStr">
         <is>
-          <t>24/36/60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K407" s="2" t="inlineStr">
@@ -39509,7 +39877,7 @@
       </c>
       <c r="J408" s="2" t="inlineStr">
         <is>
-          <t>24/36/60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K408" s="2" t="inlineStr">
@@ -39600,7 +39968,7 @@
       </c>
       <c r="J409" s="2" t="inlineStr">
         <is>
-          <t>24/36/60°</t>
+          <t>24°/36°/60°</t>
         </is>
       </c>
       <c r="K409" s="2" t="inlineStr">
@@ -40815,7 +41183,7 @@
       </c>
       <c r="J422" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K422" s="2" t="inlineStr">
@@ -40914,7 +41282,7 @@
       </c>
       <c r="J423" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K423" s="2" t="inlineStr">
@@ -41013,7 +41381,7 @@
       </c>
       <c r="J424" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K424" s="2" t="inlineStr">
@@ -41112,7 +41480,7 @@
       </c>
       <c r="J425" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K425" s="2" t="inlineStr"/>
@@ -41203,7 +41571,7 @@
       </c>
       <c r="J426" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K426" s="2" t="inlineStr"/>
@@ -41294,7 +41662,7 @@
       </c>
       <c r="J427" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K427" s="2" t="inlineStr"/>
@@ -42313,7 +42681,11 @@
       <c r="I438" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J438" s="2" t="inlineStr"/>
+      <c r="J438" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K438" s="2" t="inlineStr"/>
       <c r="L438" s="2" t="inlineStr">
         <is>
@@ -42404,7 +42776,11 @@
       <c r="I439" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J439" s="2" t="inlineStr"/>
+      <c r="J439" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K439" s="2" t="inlineStr"/>
       <c r="L439" s="2" t="inlineStr">
         <is>
@@ -42495,7 +42871,11 @@
       <c r="I440" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J440" s="2" t="inlineStr"/>
+      <c r="J440" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K440" s="2" t="inlineStr"/>
       <c r="L440" s="2" t="inlineStr">
         <is>
@@ -42586,7 +42966,11 @@
       <c r="I441" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J441" s="2" t="inlineStr"/>
+      <c r="J441" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K441" s="2" t="inlineStr"/>
       <c r="L441" s="2" t="inlineStr">
         <is>
@@ -42677,7 +43061,11 @@
       <c r="I442" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="J442" s="2" t="inlineStr"/>
+      <c r="J442" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K442" s="2" t="inlineStr"/>
       <c r="L442" s="2" t="inlineStr">
         <is>
@@ -42768,7 +43156,11 @@
       <c r="I443" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J443" s="2" t="inlineStr"/>
+      <c r="J443" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K443" s="2" t="inlineStr"/>
       <c r="L443" s="2" t="inlineStr">
         <is>
@@ -42859,7 +43251,11 @@
       <c r="I444" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J444" s="2" t="inlineStr"/>
+      <c r="J444" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K444" s="2" t="inlineStr"/>
       <c r="L444" s="2" t="inlineStr">
         <is>
@@ -42950,7 +43346,11 @@
       <c r="I445" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="J445" s="2" t="inlineStr"/>
+      <c r="J445" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K445" s="2" t="inlineStr"/>
       <c r="L445" s="2" t="inlineStr">
         <is>
@@ -43041,7 +43441,11 @@
       <c r="I446" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="J446" s="2" t="inlineStr"/>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K446" s="2" t="inlineStr"/>
       <c r="L446" s="2" t="inlineStr">
         <is>
@@ -43132,7 +43536,11 @@
       <c r="I447" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J447" s="2" t="inlineStr"/>
+      <c r="J447" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K447" s="2" t="inlineStr"/>
       <c r="L447" s="2" t="inlineStr">
         <is>
@@ -43223,7 +43631,11 @@
       <c r="I448" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J448" s="2" t="inlineStr"/>
+      <c r="J448" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K448" s="2" t="inlineStr"/>
       <c r="L448" s="2" t="inlineStr">
         <is>
@@ -43314,7 +43726,11 @@
       <c r="I449" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="J449" s="2" t="inlineStr"/>
+      <c r="J449" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K449" s="2" t="inlineStr"/>
       <c r="L449" s="2" t="inlineStr">
         <is>
@@ -43405,7 +43821,11 @@
       <c r="I450" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="J450" s="2" t="inlineStr"/>
+      <c r="J450" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K450" s="2" t="inlineStr"/>
       <c r="L450" s="2" t="inlineStr">
         <is>
@@ -43496,7 +43916,11 @@
       <c r="I451" s="5" t="n">
         <v>900</v>
       </c>
-      <c r="J451" s="2" t="inlineStr"/>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K451" s="2" t="inlineStr"/>
       <c r="L451" s="2" t="inlineStr">
         <is>
@@ -43583,7 +44007,11 @@
       <c r="I452" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="J452" s="2" t="inlineStr"/>
+      <c r="J452" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K452" s="2" t="inlineStr"/>
       <c r="L452" s="2" t="inlineStr">
         <is>
@@ -43670,7 +44098,11 @@
       <c r="I453" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J453" s="2" t="inlineStr"/>
+      <c r="J453" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K453" s="2" t="inlineStr"/>
       <c r="L453" s="2" t="inlineStr">
         <is>
@@ -43757,7 +44189,11 @@
       <c r="I454" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="J454" s="2" t="inlineStr"/>
+      <c r="J454" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K454" s="2" t="inlineStr"/>
       <c r="L454" s="2" t="inlineStr">
         <is>
@@ -43844,7 +44280,11 @@
       <c r="I455" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="J455" s="2" t="inlineStr"/>
+      <c r="J455" s="2" t="inlineStr">
+        <is>
+          <t>120°</t>
+        </is>
+      </c>
       <c r="K455" s="2" t="inlineStr"/>
       <c r="L455" s="2" t="inlineStr">
         <is>
@@ -45698,7 +46138,7 @@
       </c>
       <c r="J475" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K475" s="2" t="inlineStr">
@@ -45797,7 +46237,7 @@
       </c>
       <c r="J476" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K476" s="2" t="inlineStr">
@@ -45896,7 +46336,7 @@
       </c>
       <c r="J477" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K477" s="2" t="inlineStr">
@@ -45995,7 +46435,7 @@
       </c>
       <c r="J478" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K478" s="2" t="inlineStr">
@@ -46092,7 +46532,11 @@
       <c r="I479" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J479" s="2" t="inlineStr"/>
+      <c r="J479" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K479" s="2" t="inlineStr"/>
       <c r="L479" s="2" t="inlineStr">
         <is>
@@ -46183,7 +46627,11 @@
       <c r="I480" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J480" s="2" t="inlineStr"/>
+      <c r="J480" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K480" s="2" t="inlineStr"/>
       <c r="L480" s="2" t="inlineStr">
         <is>
@@ -46274,7 +46722,11 @@
       <c r="I481" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="J481" s="2" t="inlineStr"/>
+      <c r="J481" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K481" s="2" t="inlineStr"/>
       <c r="L481" s="2" t="inlineStr">
         <is>
@@ -46365,7 +46817,11 @@
       <c r="I482" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="J482" s="2" t="inlineStr"/>
+      <c r="J482" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K482" s="2" t="inlineStr"/>
       <c r="L482" s="2" t="inlineStr">
         <is>
@@ -46456,7 +46912,11 @@
       <c r="I483" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="J483" s="2" t="inlineStr"/>
+      <c r="J483" s="2" t="inlineStr">
+        <is>
+          <t>15°/24°/36°/55°</t>
+        </is>
+      </c>
       <c r="K483" s="2" t="inlineStr"/>
       <c r="L483" s="2" t="inlineStr">
         <is>
@@ -46549,7 +47009,7 @@
       </c>
       <c r="J484" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>30°</t>
         </is>
       </c>
       <c r="K484" s="2" t="inlineStr">
@@ -46644,7 +47104,7 @@
       </c>
       <c r="J485" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>30°</t>
         </is>
       </c>
       <c r="K485" s="2" t="inlineStr">
@@ -46739,7 +47199,7 @@
       </c>
       <c r="J486" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>30°</t>
         </is>
       </c>
       <c r="K486" s="2" t="inlineStr">
@@ -46834,7 +47294,7 @@
       </c>
       <c r="J487" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K487" s="2" t="inlineStr">
@@ -46933,7 +47393,7 @@
       </c>
       <c r="J488" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K488" s="2" t="inlineStr">
@@ -47032,7 +47492,7 @@
       </c>
       <c r="J489" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K489" s="2" t="inlineStr">
@@ -47131,7 +47591,7 @@
       </c>
       <c r="J490" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K490" s="2" t="inlineStr">
@@ -47230,7 +47690,7 @@
       </c>
       <c r="J491" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K491" s="2" t="inlineStr">
@@ -47329,7 +47789,7 @@
       </c>
       <c r="J492" s="2" t="inlineStr">
         <is>
-          <t>360°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K492" s="2" t="inlineStr">
@@ -47428,7 +47888,7 @@
       </c>
       <c r="J493" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K493" s="2" t="inlineStr">
@@ -47527,7 +47987,7 @@
       </c>
       <c r="J494" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K494" s="2" t="inlineStr">
@@ -47626,7 +48086,7 @@
       </c>
       <c r="J495" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K495" s="2" t="inlineStr">
@@ -47725,7 +48185,7 @@
       </c>
       <c r="J496" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K496" s="2" t="inlineStr">
@@ -47824,7 +48284,7 @@
       </c>
       <c r="J497" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K497" s="2" t="inlineStr">
@@ -47923,7 +48383,7 @@
       </c>
       <c r="J498" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>24°</t>
         </is>
       </c>
       <c r="K498" s="2" t="inlineStr"/>
@@ -48014,7 +48474,7 @@
       </c>
       <c r="J499" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>24°</t>
         </is>
       </c>
       <c r="K499" s="2" t="inlineStr"/>
@@ -48105,7 +48565,7 @@
       </c>
       <c r="J500" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>24°</t>
         </is>
       </c>
       <c r="K500" s="2" t="inlineStr"/>
@@ -48196,7 +48656,7 @@
       </c>
       <c r="J501" s="2" t="inlineStr">
         <is>
-          <t>350°</t>
+          <t>24°</t>
         </is>
       </c>
       <c r="K501" s="2" t="inlineStr"/>
@@ -48281,7 +48741,11 @@
       <c r="I502" s="5" t="n">
         <v>700</v>
       </c>
-      <c r="J502" s="2" t="inlineStr"/>
+      <c r="J502" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K502" s="2" t="inlineStr"/>
       <c r="L502" s="2" t="inlineStr">
         <is>
@@ -48364,7 +48828,11 @@
       <c r="I503" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="J503" s="2" t="inlineStr"/>
+      <c r="J503" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K503" s="2" t="inlineStr"/>
       <c r="L503" s="2" t="inlineStr">
         <is>
@@ -48447,7 +48915,11 @@
       <c r="I504" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="J504" s="2" t="inlineStr"/>
+      <c r="J504" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K504" s="2" t="inlineStr"/>
       <c r="L504" s="2" t="inlineStr">
         <is>
@@ -48530,7 +49002,11 @@
       <c r="I505" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="J505" s="2" t="inlineStr"/>
+      <c r="J505" s="2" t="inlineStr">
+        <is>
+          <t>24°/36°</t>
+        </is>
+      </c>
       <c r="K505" s="2" t="inlineStr"/>
       <c r="L505" s="2" t="inlineStr">
         <is>
@@ -48615,7 +49091,7 @@
       </c>
       <c r="J506" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K506" s="2" t="inlineStr">
@@ -48706,7 +49182,7 @@
       </c>
       <c r="J507" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K507" s="2" t="inlineStr">
@@ -48797,7 +49273,7 @@
       </c>
       <c r="J508" s="2" t="inlineStr">
         <is>
-          <t>15/24/36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K508" s="2" t="inlineStr">
@@ -49822,7 +50298,7 @@
       </c>
       <c r="J519" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K519" s="2" t="inlineStr">
@@ -49913,7 +50389,7 @@
       </c>
       <c r="J520" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K520" s="2" t="inlineStr">
@@ -50004,7 +50480,7 @@
       </c>
       <c r="J521" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K521" s="2" t="inlineStr">
@@ -50095,7 +50571,7 @@
       </c>
       <c r="J522" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K522" s="2" t="inlineStr">
@@ -50186,7 +50662,7 @@
       </c>
       <c r="J523" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K523" s="2" t="inlineStr">
@@ -50281,7 +50757,7 @@
       </c>
       <c r="J524" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K524" s="2" t="inlineStr"/>
@@ -50372,7 +50848,7 @@
       </c>
       <c r="J525" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K525" s="2" t="inlineStr"/>
@@ -50463,7 +50939,7 @@
       </c>
       <c r="J526" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K526" s="2" t="inlineStr"/>
@@ -50554,7 +51030,7 @@
       </c>
       <c r="J527" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K527" s="2" t="inlineStr"/>
@@ -50645,7 +51121,7 @@
       </c>
       <c r="J528" s="2" t="inlineStr">
         <is>
-          <t>110°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K528" s="2" t="inlineStr"/>
@@ -50732,7 +51208,7 @@
       </c>
       <c r="J529" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K529" s="2" t="inlineStr">
@@ -50823,7 +51299,7 @@
       </c>
       <c r="J530" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K530" s="2" t="inlineStr">
@@ -50914,7 +51390,7 @@
       </c>
       <c r="J531" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K531" s="2" t="inlineStr">
@@ -51005,7 +51481,7 @@
       </c>
       <c r="J532" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K532" s="2" t="inlineStr">
@@ -51096,7 +51572,7 @@
       </c>
       <c r="J533" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K533" s="2" t="inlineStr">
@@ -51187,7 +51663,7 @@
       </c>
       <c r="J534" s="2" t="inlineStr">
         <is>
-          <t>24/36°</t>
+          <t>24°/36°</t>
         </is>
       </c>
       <c r="K534" s="2" t="inlineStr">
@@ -53063,7 +53539,7 @@
       </c>
       <c r="J554" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K554" s="2" t="inlineStr">
@@ -53154,7 +53630,7 @@
       </c>
       <c r="J555" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K555" s="2" t="inlineStr">
@@ -53245,7 +53721,7 @@
       </c>
       <c r="J556" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K556" s="2" t="inlineStr">
@@ -53336,7 +53812,7 @@
       </c>
       <c r="J557" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K557" s="2" t="inlineStr">
@@ -53427,7 +53903,7 @@
       </c>
       <c r="J558" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K558" s="2" t="inlineStr">
@@ -53518,7 +53994,7 @@
       </c>
       <c r="J559" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K559" s="2" t="inlineStr">
@@ -53609,7 +54085,7 @@
       </c>
       <c r="J560" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K560" s="2" t="inlineStr">
@@ -53700,7 +54176,7 @@
       </c>
       <c r="J561" s="2" t="inlineStr">
         <is>
-          <t>90/120°</t>
+          <t>90°/120°</t>
         </is>
       </c>
       <c r="K561" s="2" t="inlineStr">
@@ -53791,7 +54267,7 @@
       </c>
       <c r="J562" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K562" s="2" t="inlineStr">
@@ -53882,7 +54358,7 @@
       </c>
       <c r="J563" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K563" s="2" t="inlineStr">
@@ -53973,7 +54449,7 @@
       </c>
       <c r="J564" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K564" s="2" t="inlineStr">
@@ -54064,7 +54540,7 @@
       </c>
       <c r="J565" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K565" s="2" t="inlineStr">
@@ -54155,7 +54631,7 @@
       </c>
       <c r="J566" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K566" s="2" t="inlineStr">
@@ -54246,7 +54722,7 @@
       </c>
       <c r="J567" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K567" s="2" t="inlineStr">
@@ -54333,7 +54809,7 @@
       </c>
       <c r="J568" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K568" s="2" t="inlineStr">
@@ -54420,7 +54896,7 @@
       </c>
       <c r="J569" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K569" s="2" t="inlineStr">
@@ -54507,7 +54983,7 @@
       </c>
       <c r="J570" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K570" s="2" t="inlineStr">
@@ -54594,7 +55070,7 @@
       </c>
       <c r="J571" s="2" t="inlineStr">
         <is>
-          <t>60°/90/120°</t>
+          <t>60°/90°/120°</t>
         </is>
       </c>
       <c r="K571" s="2" t="inlineStr">
@@ -54681,7 +55157,7 @@
       </c>
       <c r="J572" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*150°</t>
+          <t>60°/90°/70°/150°</t>
         </is>
       </c>
       <c r="K572" s="2" t="inlineStr">
@@ -54768,7 +55244,7 @@
       </c>
       <c r="J573" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*150°</t>
+          <t>60°/90°/70°/150°</t>
         </is>
       </c>
       <c r="K573" s="2" t="inlineStr">
@@ -54855,7 +55331,7 @@
       </c>
       <c r="J574" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*150°</t>
+          <t>60°/90°/70°/150°</t>
         </is>
       </c>
       <c r="K574" s="2" t="inlineStr">
@@ -54942,7 +55418,7 @@
       </c>
       <c r="J575" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*150°</t>
+          <t>60°/90°/70°/150°</t>
         </is>
       </c>
       <c r="K575" s="2" t="inlineStr">
@@ -55031,7 +55507,11 @@
       <c r="I576" s="11" t="n">
         <v>13000</v>
       </c>
-      <c r="J576" s="2" t="inlineStr"/>
+      <c r="J576" s="2" t="inlineStr">
+        <is>
+          <t>T2/T3/T4</t>
+        </is>
+      </c>
       <c r="K576" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -55122,7 +55602,11 @@
       <c r="I577" s="11" t="n">
         <v>19500</v>
       </c>
-      <c r="J577" s="2" t="inlineStr"/>
+      <c r="J577" s="2" t="inlineStr">
+        <is>
+          <t>T2/T3/T4</t>
+        </is>
+      </c>
       <c r="K577" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -55213,7 +55697,11 @@
       <c r="I578" s="11" t="n">
         <v>26000</v>
       </c>
-      <c r="J578" s="2" t="inlineStr"/>
+      <c r="J578" s="2" t="inlineStr">
+        <is>
+          <t>T2/T3/T4</t>
+        </is>
+      </c>
       <c r="K578" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -55304,7 +55792,11 @@
       <c r="I579" s="11" t="n">
         <v>31200</v>
       </c>
-      <c r="J579" s="2" t="inlineStr"/>
+      <c r="J579" s="2" t="inlineStr">
+        <is>
+          <t>T2/T3/T4</t>
+        </is>
+      </c>
       <c r="K579" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -55395,7 +55887,11 @@
       <c r="I580" s="11" t="n">
         <v>39000</v>
       </c>
-      <c r="J580" s="2" t="inlineStr"/>
+      <c r="J580" s="2" t="inlineStr">
+        <is>
+          <t>T2/T3/T4</t>
+        </is>
+      </c>
       <c r="K580" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -55832,7 +56328,7 @@
       </c>
       <c r="J585" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*130°</t>
+          <t>60°/90°/70°/130°</t>
         </is>
       </c>
       <c r="K585" s="2" t="inlineStr">
@@ -55923,7 +56419,7 @@
       </c>
       <c r="J586" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*130°</t>
+          <t>60°/90°/70°/130°</t>
         </is>
       </c>
       <c r="K586" s="2" t="inlineStr">
@@ -56014,7 +56510,7 @@
       </c>
       <c r="J587" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*130°</t>
+          <t>60°/90°/70°/130°</t>
         </is>
       </c>
       <c r="K587" s="2" t="inlineStr">
@@ -56105,7 +56601,7 @@
       </c>
       <c r="J588" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*130°</t>
+          <t>60°/90°/70°/130°</t>
         </is>
       </c>
       <c r="K588" s="2" t="inlineStr">
@@ -56196,7 +56692,7 @@
       </c>
       <c r="J589" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/70°*130°</t>
+          <t>60°/90°/70°/130°</t>
         </is>
       </c>
       <c r="K589" s="2" t="inlineStr">
@@ -56291,7 +56787,7 @@
       </c>
       <c r="J590" s="2" t="inlineStr">
         <is>
-          <t>140°</t>
+          <t>70*140°/110°</t>
         </is>
       </c>
       <c r="K590" s="2" t="inlineStr">
@@ -56382,7 +56878,7 @@
       </c>
       <c r="J591" s="2" t="inlineStr">
         <is>
-          <t>140°</t>
+          <t>70*140°/110°</t>
         </is>
       </c>
       <c r="K591" s="2" t="inlineStr">
@@ -56473,7 +56969,7 @@
       </c>
       <c r="J592" s="2" t="inlineStr">
         <is>
-          <t>140°</t>
+          <t>70*140°/110°</t>
         </is>
       </c>
       <c r="K592" s="2" t="inlineStr">
@@ -56564,7 +57060,7 @@
       </c>
       <c r="J593" s="2" t="inlineStr">
         <is>
-          <t>140°</t>
+          <t>70*140°/110°</t>
         </is>
       </c>
       <c r="K593" s="2" t="inlineStr">
@@ -56651,7 +57147,7 @@
       </c>
       <c r="J594" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/120°/T2</t>
+          <t>60°/90°/120°/T2/T3/T4</t>
         </is>
       </c>
       <c r="K594" s="2" t="inlineStr"/>
@@ -56730,7 +57226,7 @@
       </c>
       <c r="J595" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/120°/T2</t>
+          <t>60°/90°/120°/T2/T3/T4</t>
         </is>
       </c>
       <c r="K595" s="2" t="inlineStr"/>
@@ -56809,7 +57305,7 @@
       </c>
       <c r="J596" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/120°/T2</t>
+          <t>60°/90°/120°/T2/T3/T4</t>
         </is>
       </c>
       <c r="K596" s="2" t="inlineStr"/>
@@ -56888,7 +57384,7 @@
       </c>
       <c r="J597" s="2" t="inlineStr">
         <is>
-          <t>60°/90°/120°/T2</t>
+          <t>60°/90°/120°/T2/T3/T4</t>
         </is>
       </c>
       <c r="K597" s="2" t="inlineStr"/>
@@ -59040,7 +59536,7 @@
       </c>
       <c r="J621" s="2" t="inlineStr">
         <is>
-          <t>90°</t>
+          <t>90°/75*145°</t>
         </is>
       </c>
       <c r="K621" s="2" t="inlineStr">
@@ -59131,7 +59627,7 @@
       </c>
       <c r="J622" s="2" t="inlineStr">
         <is>
-          <t>90°</t>
+          <t>90°/75*145°</t>
         </is>
       </c>
       <c r="K622" s="2" t="inlineStr">
@@ -59222,7 +59718,7 @@
       </c>
       <c r="J623" s="2" t="inlineStr">
         <is>
-          <t>90°</t>
+          <t>90°/75*145°</t>
         </is>
       </c>
       <c r="K623" s="2" t="inlineStr">
@@ -59313,7 +59809,7 @@
       </c>
       <c r="J624" s="2" t="inlineStr">
         <is>
-          <t>90°</t>
+          <t>90°/75*145°</t>
         </is>
       </c>
       <c r="K624" s="2" t="inlineStr">
@@ -59404,7 +59900,7 @@
       </c>
       <c r="J625" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K625" s="2" t="inlineStr">
@@ -59495,7 +59991,7 @@
       </c>
       <c r="J626" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K626" s="2" t="inlineStr">
@@ -59586,7 +60082,7 @@
       </c>
       <c r="J627" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K627" s="2" t="inlineStr">
@@ -59677,7 +60173,7 @@
       </c>
       <c r="J628" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K628" s="2" t="inlineStr">
@@ -59768,7 +60264,7 @@
       </c>
       <c r="J629" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K629" s="2" t="inlineStr">
@@ -59859,7 +60355,7 @@
       </c>
       <c r="J630" s="2" t="inlineStr">
         <is>
-          <t>25/45/60/90°</t>
+          <t>25°/45°/60°/90°</t>
         </is>
       </c>
       <c r="K630" s="2" t="inlineStr">
@@ -59940,7 +60436,7 @@
       <c r="I631" s="11" t="n"/>
       <c r="J631" s="2" t="inlineStr">
         <is>
-          <t>60°</t>
+          <t>60°/95°</t>
         </is>
       </c>
       <c r="K631" s="2" t="inlineStr">
@@ -60017,7 +60513,7 @@
       <c r="I632" s="11" t="n"/>
       <c r="J632" s="2" t="inlineStr">
         <is>
-          <t>60°</t>
+          <t>60°/95°</t>
         </is>
       </c>
       <c r="K632" s="2" t="inlineStr">
@@ -60094,7 +60590,7 @@
       <c r="I633" s="11" t="n"/>
       <c r="J633" s="2" t="inlineStr">
         <is>
-          <t>60°</t>
+          <t>60°/95°</t>
         </is>
       </c>
       <c r="K633" s="2" t="inlineStr">
@@ -60171,7 +60667,7 @@
       <c r="I634" s="11" t="n"/>
       <c r="J634" s="2" t="inlineStr">
         <is>
-          <t>60°</t>
+          <t>60°/95°</t>
         </is>
       </c>
       <c r="K634" s="2" t="inlineStr">
@@ -60248,7 +60744,7 @@
       <c r="I635" s="10" t="n"/>
       <c r="J635" s="6" t="inlineStr">
         <is>
-          <t>60°</t>
+          <t>60°/95°</t>
         </is>
       </c>
       <c r="K635" s="6" t="inlineStr">
@@ -69609,7 +70105,11 @@
       <c r="I752" s="11" t="n">
         <v>16500</v>
       </c>
-      <c r="J752" s="2" t="inlineStr"/>
+      <c r="J752" s="2" t="inlineStr">
+        <is>
+          <t>90°</t>
+        </is>
+      </c>
       <c r="K752" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -69688,7 +70188,11 @@
       <c r="I753" s="11" t="n">
         <v>16500</v>
       </c>
-      <c r="J753" s="2" t="inlineStr"/>
+      <c r="J753" s="2" t="inlineStr">
+        <is>
+          <t>90°</t>
+        </is>
+      </c>
       <c r="K753" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -69767,7 +70271,11 @@
       <c r="I754" s="11" t="n">
         <v>16500</v>
       </c>
-      <c r="J754" s="2" t="inlineStr"/>
+      <c r="J754" s="2" t="inlineStr">
+        <is>
+          <t>90°</t>
+        </is>
+      </c>
       <c r="K754" s="2" t="inlineStr">
         <is>
           <t>IP65</t>
@@ -71069,7 +71577,7 @@
       </c>
       <c r="J770" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K770" s="2" t="inlineStr"/>
@@ -71156,7 +71664,7 @@
       </c>
       <c r="J771" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K771" s="2" t="inlineStr"/>
@@ -71243,7 +71751,7 @@
       </c>
       <c r="J772" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K772" s="2" t="inlineStr"/>
@@ -72548,7 +73056,7 @@
       </c>
       <c r="J787" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K787" s="2" t="inlineStr"/>
@@ -72635,7 +73143,7 @@
       </c>
       <c r="J788" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K788" s="2" t="inlineStr"/>
@@ -72722,7 +73230,7 @@
       </c>
       <c r="J789" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K789" s="2" t="inlineStr"/>
@@ -72809,7 +73317,7 @@
       </c>
       <c r="J790" s="2" t="inlineStr">
         <is>
-          <t>36°</t>
+          <t>15°/24°/36°</t>
         </is>
       </c>
       <c r="K790" s="2" t="inlineStr"/>

</xml_diff>